<commit_message>
Brought 2 other pages plus a fix
Automated migration updates generated by Experience Modernization Agent.

Changed files (10):
- templates/procedure-detail/procedure-detail.css
- tools/importer/import-procedure-detail.bundle.js
- tools/importer/reports/import-procedure-detail.report.xlsx
- tools/importer/reports/us/en/ivs/treatments/bone-tumor-ablation.report.json
- tools/importer/reports/us/en/ivs/treatments/radiofrequency-ablation.report.json
- tools/importer/reports/us/en/ivs/treatments/sacroplasty.report.json
- tools/importer/transformers/procedure-detail/procedure-detail-cleanup.js
- tools/importer/urls-procedure-detail.txt
- tools/style-validator/configs/procedure-detail.json
- tools/style-validator/lib/extract.js
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-procedure-detail.report.xlsx
+++ b/tools/importer/reports/import-procedure-detail.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="70">
   <si>
     <t>_reportFile</t>
   </si>
@@ -131,6 +131,21 @@
     <t>Balloon kyphoplasty | Interventional Spine | Stryker</t>
   </si>
   <si>
+    <t>us/en/ivs/treatments/bone-tumor-ablation.report.json</t>
+  </si>
+  <si>
+    <t>us/en/ivs/treatments/bone-tumor-ablation</t>
+  </si>
+  <si>
+    <t>2026-09-09T09:44:37.928Z</t>
+  </si>
+  <si>
+    <t>Bone tumor ablation | Interventional Spine | Stryker</t>
+  </si>
+  <si>
+    <t>https://patients.stryker.com/us/en/ivs/treatments/bone-tumor-ablation.html</t>
+  </si>
+  <si>
     <t>us/en/ivs/treatments/disc-decompression.report.json</t>
   </si>
   <si>
@@ -152,13 +167,31 @@
     <t>us/en/ivs/treatments/radiofrequency-ablation</t>
   </si>
   <si>
-    <t>2026-09-08T07:05:53.479Z</t>
+    <t>2026-09-09T08:18:43.313Z</t>
   </si>
   <si>
     <t>Radiofrequency ablation | Interventional Spine | Stryker</t>
   </si>
   <si>
     <t>https://patients.stryker.com/us/en/ivs/treatments/radiofrequency-ablation.html</t>
+  </si>
+  <si>
+    <t>us/en/ivs/treatments/sacroplasty.report.json</t>
+  </si>
+  <si>
+    <t>["hero","panel-cta","panel-dark","panel-dark","cards","panel-gold"]</t>
+  </si>
+  <si>
+    <t>us/en/ivs/treatments/sacroplasty</t>
+  </si>
+  <si>
+    <t>2026-09-09T09:44:53.028Z</t>
+  </si>
+  <si>
+    <t>Sacroplasty | Interventional Spine | Stryker</t>
+  </si>
+  <si>
+    <t>https://patients.stryker.com/us/en/ivs/treatments/sacroplasty.html</t>
   </si>
   <si>
     <t>us/en/ivs/treatments/spinejack-system.report.json</t>
@@ -580,7 +613,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J9"/>
+  <dimension ref="A1:J11"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="4" width="50" customWidth="1"/>
@@ -878,6 +911,70 @@
         <v>58</v>
       </c>
     </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>59</v>
+      </c>
+      <c r="B10" t="s">
+        <v>33</v>
+      </c>
+      <c r="C10" t="s">
+        <v>12</v>
+      </c>
+      <c r="D10" t="s">
+        <v>12</v>
+      </c>
+      <c r="E10" t="s">
+        <v>60</v>
+      </c>
+      <c r="F10" t="s">
+        <v>14</v>
+      </c>
+      <c r="G10" t="s">
+        <v>35</v>
+      </c>
+      <c r="H10" t="s">
+        <v>61</v>
+      </c>
+      <c r="I10" t="s">
+        <v>62</v>
+      </c>
+      <c r="J10" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>64</v>
+      </c>
+      <c r="B11" t="s">
+        <v>65</v>
+      </c>
+      <c r="C11" t="s">
+        <v>12</v>
+      </c>
+      <c r="D11" t="s">
+        <v>12</v>
+      </c>
+      <c r="E11" t="s">
+        <v>66</v>
+      </c>
+      <c r="F11" t="s">
+        <v>14</v>
+      </c>
+      <c r="G11" t="s">
+        <v>35</v>
+      </c>
+      <c r="H11" t="s">
+        <v>67</v>
+      </c>
+      <c r="I11" t="s">
+        <v>68</v>
+      </c>
+      <c r="J11" t="s">
+        <v>69</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:J1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>